<commit_message>
let matrixTests, multiScore, GSEABase, STRINGdb and openxlsx do the jobs my own loops were doing
</commit_message>
<xml_diff>
--- a/04_Networks/03_Classify_Associate/c_data/module_screens.xlsx
+++ b/04_Networks/03_Classify_Associate/c_data/module_screens.xlsx
@@ -2768,7 +2768,7 @@
         <v>6</v>
       </c>
       <c r="E2" t="n">
-        <v>0.555555555555555</v>
+        <v>0.555555555555556</v>
       </c>
       <c r="F2" t="n">
         <v>0.529368106184798</v>
@@ -2837,7 +2837,7 @@
         <v>6</v>
       </c>
       <c r="E5" t="n">
-        <v>0.555555555555555</v>
+        <v>0.555555555555556</v>
       </c>
       <c r="F5" t="n">
         <v>0.833935414088552</v>
@@ -3024,10 +3024,10 @@
         <v>0.916666666666667</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0360316862182335</v>
+        <v>0.0360316862182336</v>
       </c>
       <c r="G13" t="n">
-        <v>0.432380234618802</v>
+        <v>0.432380234618803</v>
       </c>
     </row>
     <row r="14">
@@ -3320,7 +3320,7 @@
         <v>7</v>
       </c>
       <c r="E26" t="n">
-        <v>0.571428571428572</v>
+        <v>0.571428571428571</v>
       </c>
       <c r="F26" t="n">
         <v>0.799846105662473</v>
@@ -3369,7 +3369,7 @@
         <v>0.673469387755102</v>
       </c>
       <c r="F28" t="n">
-        <v>0.204893893816378</v>
+        <v>0.204893893816379</v>
       </c>
       <c r="G28" t="n">
         <v>0.351246675113792</v>
@@ -3435,7 +3435,7 @@
         <v>7</v>
       </c>
       <c r="E31" t="n">
-        <v>0.918367346938775</v>
+        <v>0.918367346938776</v>
       </c>
       <c r="F31" t="n">
         <v>0.0519129649350183</v>
@@ -3553,7 +3553,7 @@
         <v>0.612244897959184</v>
       </c>
       <c r="F36" t="n">
-        <v>0.204893893816378</v>
+        <v>0.204893893816379</v>
       </c>
       <c r="G36" t="n">
         <v>0.351246675113792</v>
@@ -3875,7 +3875,7 @@
         <v>0.535714285714286</v>
       </c>
       <c r="F50" t="n">
-        <v>0.862186694400763</v>
+        <v>0.862186694400762</v>
       </c>
       <c r="G50" t="n">
         <v>0.94056730298265</v>
@@ -3944,7 +3944,7 @@
         <v>0.553571428571429</v>
       </c>
       <c r="F53" t="n">
-        <v>0.772337441292781</v>
+        <v>0.77233744129278</v>
       </c>
       <c r="G53" t="n">
         <v>0.94056730298265</v>
@@ -3990,7 +3990,7 @@
         <v>0.535714285714286</v>
       </c>
       <c r="F55" t="n">
-        <v>0.862186694400763</v>
+        <v>0.862186694400762</v>
       </c>
       <c r="G55" t="n">
         <v>0.94056730298265</v>
@@ -4151,7 +4151,7 @@
         <v>0.541666666666667</v>
       </c>
       <c r="F62" t="n">
-        <v>0.84645059687659</v>
+        <v>0.846450596876591</v>
       </c>
       <c r="G62" t="n">
         <v>1</v>
@@ -4611,7 +4611,7 @@
         <v>0.785714285714286</v>
       </c>
       <c r="F82" t="n">
-        <v>0.0728488583209921</v>
+        <v>0.072848858320992</v>
       </c>
       <c r="G82" t="n">
         <v>0.373350188712092</v>
@@ -4654,7 +4654,7 @@
         <v>7</v>
       </c>
       <c r="E84" t="n">
-        <v>0.678571428571428</v>
+        <v>0.678571428571429</v>
       </c>
       <c r="F84" t="n">
         <v>0.271588674243375</v>
@@ -15220,7 +15220,7 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0.432380234618802</v>
+        <v>0.432380234618803</v>
       </c>
     </row>
     <row r="3">

</xml_diff>